<commit_message>
Prune duplicate TC block in Đăng tin, sync BRD v3.2 scenario updates, add colleague CA analysis draft
- Remove 4 duplicate TCs (TC_04.110-113, "Trang chủ, Hoạt động — Tin tự động Hết hạn") from Đăng tin, already covered in TC-HOATDONG (175→171 TC total)
- Sync MASTER-MEMORY/CHANGELOG/version MEMORY logs for the prune
- Pull in latest scenario/requirement/review updates (BRD v3.2, team merge prep with anhdc4)
- Add colleague's draft analysis + test cases folder for upcoming project merge

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_test-cases/v1.0/fragments/TC-CANHAN-v1.0.xlsx
+++ b/03_test-cases/v1.0/fragments/TC-CANHAN-v1.0.xlsx
@@ -3471,7 +3471,7 @@
       </c>
       <c r="C18" s="205" t="inlineStr">
         <is>
-          <t>Quan sát thực tế app</t>
+          <t>DOC-v1.0-02 §3.9</t>
         </is>
       </c>
       <c r="D18" s="205" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="C19" s="229" t="inlineStr">
         <is>
-          <t>Quan sát thực tế app</t>
+          <t>DOC-v1.0-01 (GIFT-01) + ảnh DOC-v1.0-04</t>
         </is>
       </c>
       <c r="D19" s="229" t="inlineStr">
@@ -3877,7 +3877,7 @@
       </c>
       <c r="C23" s="229" t="inlineStr">
         <is>
-          <t>Quan sát thực tế app</t>
+          <t>Ảnh DOC-v1.0-04 (Quà đã nhận)</t>
         </is>
       </c>
       <c r="D23" s="229" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C24" s="229" t="inlineStr">
         <is>
-          <t>Quan sát thực tế app</t>
+          <t>Ảnh DOC-v1.0-04 (Quà đã nhận)</t>
         </is>
       </c>
       <c r="D24" s="229" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="C25" s="205" t="inlineStr">
         <is>
-          <t>Quan sát thực tế app</t>
+          <t>Chờ BA bổ sung</t>
         </is>
       </c>
       <c r="D25" s="205" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C26" s="229" t="inlineStr">
         <is>
-          <t>Quan sát thực tế app</t>
+          <t>Chờ BA bổ sung</t>
         </is>
       </c>
       <c r="D26" s="229" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="C27" s="229" t="inlineStr">
         <is>
-          <t>Quan sát thực tế app</t>
+          <t>Chờ BA bổ sung</t>
         </is>
       </c>
       <c r="D27" s="229" t="inlineStr">

</xml_diff>